<commit_message>
Update soccer trades 2026-08-11 20:03:02 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/FA Cup England/trades.xlsx
+++ b/data/sxbet/ligas/FA Cup England/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xa0f8e864c3790e0b04279f595cd2b6256076aae2d5cb0653cf1c7d3818da77a6</t>
+          <t>0x5280fa1e8d6de44c7914cb4eb06f5cb04b2bcf5a22baa51e4e335978ef409473</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>12.97997</t>
+          <t>8.16999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7825</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x3a78b8f99779adbd9e98e2e6eab392c9d1ce2c8336e5cb1caece466b178bf3ab</t>
+          <t>0x58ce427771a4747942dba5d0b61c2976c834540fc4bf96c0add242cd6c115aee</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786457562</t>
+          <t>1786473900</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>16.587821</t>
+          <t>13.230753</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x52a7fcd3920570261f5a16eb304eddc2d668c08ad563042cb4e41659646fa2dd</t>
+          <t>0x1e35e28c6d26caa2fbc05eafb4824258a3ed9e6efbc34d2a13b9d6a6b99c1bab</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,94 +643,86 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17.24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.3962</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mossley AFC vs Silsden</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Mossley AFC</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Silsden</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xc1eb934b4da4af416075dd27e12ab004a24c884d01e4fe0f758a94ff25ab7015</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19766919</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0.00249</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.645</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Kingstonian</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>FA Cup England</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Kingstonian vs Hastings United</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Kingstonian</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Hastings United</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19718588</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786131380</t>
+          <t>1786473312</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786128300</t>
+          <t>1786473900</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>0.00386</t>
+          <t>43.507886</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x1a7f9c36ef037446acb729c4aa4b82309312cfa92208667128e6f99321df4af3</t>
+          <t>0x1b24cd8e3f0e2cb21aa61e8f0d6c1ef0d3db1ac2f4f98bd9204322e433d2356f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -762,22 +754,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>102.78</t>
+          <t>17.34999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5875</t>
+          <t>1.6225</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>FA Cup England</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Kingstonian</t>
+          <t>Mossley AFC</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -787,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Kingstonian vs Hastings United</t>
+          <t>Mossley AFC vs Silsden</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Kingstonian</t>
+          <t>Mossley AFC</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Hastings United</t>
+          <t>Silsden</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+          <t>0xc1eb934b4da4af416075dd27e12ab004a24c884d01e4fe0f758a94ff25ab7015</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19718588</t>
+          <t>L19766919</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786131367</t>
+          <t>1786473226</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786128300</t>
+          <t>1786473900</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>174.944681</t>
+          <t>27.87147</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x49acf03cf8812b8213b89dd52064fde8bac878e692008a60c3372c3951d2b712</t>
+          <t>0x255d243aa4448d42eb1c138a144e082bae6733c497d4d7df7f2970d0796100b8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -867,23 +859,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>156.31</t>
+          <t>4.41999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.6663</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>FA Cup England</t>
@@ -891,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Kingstonian vs Hastings United</t>
+          <t>Mossley AFC vs Silsden</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Kingstonian</t>
+          <t>Mossley AFC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Hastings United</t>
+          <t>Silsden</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+          <t>0xe413b3f2bfa9b50149089dee4c1368189d76c84d20ddd0f3eef933c38b2eba68</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19718588</t>
+          <t>L19766919</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786131009</t>
+          <t>1786473225</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786128300</t>
+          <t>1786473900</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>284.2</t>
+          <t>6.634131</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,102 +963,94 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x6fe66db5744d90337799e26ebe4b2167deaf50f2214378a04d3f33ce33b9bd6d</t>
+          <t>0xa0f8e864c3790e0b04279f595cd2b6256076aae2d5cb0653cf1c7d3818da77a6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x62f30772266D06e1468de3b73416006613793F89</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12.97997</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.7825</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mossley AFC vs Silsden</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mossley AFC</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Silsden</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x3a78b8f99779adbd9e98e2e6eab392c9d1ce2c8336e5cb1caece466b178bf3ab</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19766919</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2.26</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1.4412</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Kingstonian</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>FA Cup England</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Kingstonian vs Hastings United</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Kingstonian</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Hastings United</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>L19718588</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786108854</t>
+          <t>1786457562</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786128300</t>
+          <t>1786473900</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>5.121813</t>
+          <t>16.587821</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,110 +1067,550 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>0x52a7fcd3920570261f5a16eb304eddc2d668c08ad563042cb4e41659646fa2dd</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.00249</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.645</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Kingstonian vs Hastings United</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Hastings United</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19718588</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786131380</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0.00386</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x1a7f9c36ef037446acb729c4aa4b82309312cfa92208667128e6f99321df4af3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>102.78</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.5875</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Kingstonian vs Hastings United</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Hastings United</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19718588</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786131367</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>174.944681</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x49acf03cf8812b8213b89dd52064fde8bac878e692008a60c3372c3951d2b712</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>156.31</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Kingstonian vs Hastings United</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Hastings United</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19718588</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786131009</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>284.2</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x6fe66db5744d90337799e26ebe4b2167deaf50f2214378a04d3f33ce33b9bd6d</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0x62f30772266D06e1468de3b73416006613793F89</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2.26</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.4412</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FA Cup England</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Kingstonian vs Hastings United</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Kingstonian</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Hastings United</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19718588</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786108854</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>5.121813</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>0x78624edc9adf7b0e4c4d4036f7e28d75b883bf617d8c603636db4118e2de1309</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>0x62f30772266D06e1468de3b73416006613793F89</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>2.26</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>1.4425</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Kingstonian</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>FA Cup England</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Kingstonian vs Hastings United</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Kingstonian</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Hastings United</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>0x7514670cd8b9a0dfc860e92bddfba35e407f914f1a88a19a52848f51ccad6fe0</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>L19718588</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>1786108249</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>1786128300</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>5.107345</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>